<commit_message>
Update posts.xlsx after post
</commit_message>
<xml_diff>
--- a/posts.xlsx
+++ b/posts.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C843"/>
+  <dimension ref="A1:C842"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -17890,46 +17890,25 @@
     <row r="833">
       <c r="A833" t="inlineStr">
         <is>
-          <t xml:space="preserve">「気分が良いぞう」I فيل GOOD
-アイ・フィール・グッド [ai fiyl gud]
-⁦「象」フィール ( فيل )[fiyl]：英語「感じる」feel：( فـ )[f-]・( ـيـ )[-y-]・( ـل )[-l]：( ف )[f]・( ي )[y]・( ل )[l]⁩
-気分（キブン）・良い（いい／よい）
-2308 出典不明 </t>
-        </is>
-      </c>
-      <c r="B833" t="inlineStr">
-        <is>
-          <t>images/「気分が良いぞう」_img1.jpg</t>
-        </is>
-      </c>
-      <c r="C833" t="inlineStr">
-        <is>
-          <t>洒落 ,和訳</t>
-        </is>
-      </c>
-    </row>
-    <row r="834">
-      <c r="A834" t="inlineStr">
-        <is>
           <t xml:space="preserve">「ようこそ」اهلا وسهلا
 アハラン・ワサハラン ['ahlan wa-sahlan]
 ⁦( أَ )['a]・( هـ )[h-]・( ـلاً )[-lan]・( سـ )[s-]・( ـهـ )[-h-]⁩
 2106 behance Anwar Al Eissa </t>
         </is>
       </c>
-      <c r="B834" t="inlineStr">
+      <c r="B833" t="inlineStr">
         <is>
           <t>images/「ようこそ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C834" t="inlineStr">
+      <c r="C833" t="inlineStr">
         <is>
           <t>アラビア語</t>
         </is>
       </c>
     </row>
-    <row r="835">
-      <c r="A835" t="inlineStr">
+    <row r="834">
+      <c r="A834" t="inlineStr">
         <is>
           <t xml:space="preserve">「まぁ何というサプライズでしょう」
 يا لها من مفاجأة
@@ -17940,19 +17919,19 @@
 2108 neelwafurat com </t>
         </is>
       </c>
-      <c r="B835" t="inlineStr">
+      <c r="B834" t="inlineStr">
         <is>
           <t>images/「まぁ何というサプライズでしょう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C835" t="inlineStr">
+      <c r="C834" t="inlineStr">
         <is>
           <t>中国語 ,学習</t>
         </is>
       </c>
     </row>
-    <row r="836">
-      <c r="A836" t="inlineStr">
+    <row r="835">
+      <c r="A835" t="inlineStr">
         <is>
           <t xml:space="preserve">「ハックション」اتشوو
 アチュー！ ['aatShuu]
@@ -17960,19 +17939,19 @@
 1811 </t>
         </is>
       </c>
-      <c r="B836" t="inlineStr">
+      <c r="B835" t="inlineStr">
         <is>
           <t>images/「ハックション」_img1.jpg</t>
         </is>
       </c>
-      <c r="C836" t="inlineStr">
+      <c r="C835" t="inlineStr">
         <is>
           <t>あらびあや</t>
         </is>
       </c>
     </row>
-    <row r="837">
-      <c r="A837" t="inlineStr">
+    <row r="836">
+      <c r="A836" t="inlineStr">
         <is>
           <t xml:space="preserve">「スブハーナッラー」「アルハムドゥリッラー」「アッラーアクバル」
 سبحان الله
@@ -17983,19 +17962,19 @@
 2308 dribbble com </t>
         </is>
       </c>
-      <c r="B837" t="inlineStr">
+      <c r="B836" t="inlineStr">
         <is>
           <t>images/「スブハーナッラー」「アルハムドゥリッ_img1.jpg</t>
         </is>
       </c>
-      <c r="C837" t="inlineStr">
+      <c r="C836" t="inlineStr">
         <is>
           <t>四角 ,コンパクト</t>
         </is>
       </c>
     </row>
-    <row r="838">
-      <c r="A838" t="inlineStr">
+    <row r="837">
+      <c r="A837" t="inlineStr">
         <is>
           <t xml:space="preserve">「すごく美味しい！」لذيذ جدًا
 ラズィーズ・ジッダン [laDhiiDh jiddan]
@@ -18004,19 +17983,19 @@
 2109 goodreads com </t>
         </is>
       </c>
-      <c r="B838" t="inlineStr">
+      <c r="B837" t="inlineStr">
         <is>
           <t>images/「すごく美味しい！」_img1.jpg</t>
         </is>
       </c>
-      <c r="C838" t="inlineStr">
+      <c r="C837" t="inlineStr">
         <is>
           <t>フレーズ ,感想</t>
         </is>
       </c>
     </row>
-    <row r="839">
-      <c r="A839" t="inlineStr">
+    <row r="838">
+      <c r="A838" t="inlineStr">
         <is>
           <t xml:space="preserve">「しとしと、雨」تك تك يا مطر
 ティクティク [tik tik yaa ma_tar]
@@ -18025,19 +18004,19 @@
 2308 出典不明 </t>
         </is>
       </c>
-      <c r="B839" t="inlineStr">
+      <c r="B838" t="inlineStr">
         <is>
           <t>images/「しとしと、雨」_img1.jpg</t>
         </is>
       </c>
-      <c r="C839" t="inlineStr">
+      <c r="C838" t="inlineStr">
         <is>
           <t>天気 ,梅雨</t>
         </is>
       </c>
     </row>
-    <row r="840">
-      <c r="A840" t="inlineStr">
+    <row r="839">
+      <c r="A839" t="inlineStr">
         <is>
           <t xml:space="preserve">「さかさま」رأساً على عقب
 ラッアサン・アラー・アケブ [ra'san *alaa *aqib]
@@ -18045,19 +18024,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B840" t="inlineStr">
+      <c r="B839" t="inlineStr">
         <is>
           <t>images/「さかさま」_img1.jpg</t>
         </is>
       </c>
-      <c r="C840" t="inlineStr">
+      <c r="C839" t="inlineStr">
         <is>
           <t>壁 ,上下</t>
         </is>
       </c>
     </row>
-    <row r="841">
-      <c r="A841" t="inlineStr">
+    <row r="840">
+      <c r="A840" t="inlineStr">
         <is>
           <t xml:space="preserve">「エジプトよどこへ行った」
 فينك يا مصر؟
@@ -18067,19 +18046,19 @@
 1809 shehabfawzy1.tumblr </t>
         </is>
       </c>
-      <c r="B841" t="inlineStr">
+      <c r="B840" t="inlineStr">
         <is>
           <t>images/「エジプトよどこへ行った」_img1.jpg</t>
         </is>
       </c>
-      <c r="C841" t="inlineStr">
+      <c r="C840" t="inlineStr">
         <is>
           <t>ピラミッド ,歴史</t>
         </is>
       </c>
     </row>
-    <row r="842">
-      <c r="A842" t="inlineStr">
+    <row r="841">
+      <c r="A841" t="inlineStr">
         <is>
           <t xml:space="preserve">「ありがとう」شكراً
 シュクラン [Shukran]
@@ -18087,19 +18066,19 @@
 2109 出典不明 </t>
         </is>
       </c>
-      <c r="B842" t="inlineStr">
+      <c r="B841" t="inlineStr">
         <is>
           <t>images/「ありがとう」_img1.jpg</t>
         </is>
       </c>
-      <c r="C842" t="inlineStr">
+      <c r="C841" t="inlineStr">
         <is>
           <t>挨拶 ,文字</t>
         </is>
       </c>
     </row>
-    <row r="843">
-      <c r="A843" t="inlineStr">
+    <row r="842">
+      <c r="A842" t="inlineStr">
         <is>
           <t xml:space="preserve">「昼寝の時間だ」
 إنه وقت القيلولة
@@ -18108,12 +18087,12 @@
 2501 https://x.com/NatGeoMagArab/status/1858049951579910486 </t>
         </is>
       </c>
-      <c r="B843" t="inlineStr">
+      <c r="B842" t="inlineStr">
         <is>
           <t>images/「昼寝の時間だ」_img1.jpg</t>
         </is>
       </c>
-      <c r="C843" t="inlineStr">
+      <c r="C842" t="inlineStr">
         <is>
           <t>手書き語学 ,アラビア語 ,ペンギン</t>
         </is>

</xml_diff>